<commit_message>
updated DCR and started on block diagram
</commit_message>
<xml_diff>
--- a/ADCS/DesignCriteriaReview.xlsx
+++ b/ADCS/DesignCriteriaReview.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Main Engineering\Engineering\Project Genesis EE Notes\ADCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D3299B-239C-47C2-9BA4-2AA8526DE134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB10F90-359D-497F-89DD-E5D1F067EBE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Design Criteria" sheetId="1" r:id="rId1"/>
+    <sheet name="Used Mezz Pins" sheetId="2" r:id="rId2"/>
+    <sheet name="Electrical Interfaces" sheetId="3" r:id="rId3"/>
+    <sheet name="Block Diagram" sheetId="4" r:id="rId4"/>
+    <sheet name="Startracker" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,10 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
-  <si>
-    <t>Requirement</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
   <si>
     <t>Specification</t>
   </si>
@@ -97,6 +98,111 @@
   </si>
   <si>
     <t>relatively arbitrary but should definitly be sufficient to hit pointing req</t>
+  </si>
+  <si>
+    <t>Used Digital Mezz Pins</t>
+  </si>
+  <si>
+    <t>Used Analog Mezz Pins</t>
+  </si>
+  <si>
+    <t>Power Off Pin</t>
+  </si>
+  <si>
+    <t>Batt Raw (13-16V)</t>
+  </si>
+  <si>
+    <t>CAN_H</t>
+  </si>
+  <si>
+    <t>5V</t>
+  </si>
+  <si>
+    <t>CAN_L</t>
+  </si>
+  <si>
+    <t>3V3</t>
+  </si>
+  <si>
+    <t>Functional Requirements</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>ADCS</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>Thermal</t>
+  </si>
+  <si>
+    <t>Mechanical</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Board outline 80x80mm</t>
+  </si>
+  <si>
+    <t>Harnessing</t>
+  </si>
+  <si>
+    <t>Full Power Shutoff</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Fault Tolerance</t>
+  </si>
+  <si>
+    <t>1FT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thermal Dissipation Requirements </t>
+  </si>
+  <si>
+    <t>&lt;XXW</t>
+  </si>
+  <si>
+    <t>Fault tolerance to mission failure</t>
+  </si>
+  <si>
+    <t>IMU Accuracy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is +-10DEG  </t>
+  </si>
+  <si>
+    <t>Allow OBC to fully shutdown board with loadswitch to alllow for a hard power cycle</t>
+  </si>
+  <si>
+    <t>Non Volatile Storage</t>
+  </si>
+  <si>
+    <t>Temperature Sense</t>
+  </si>
+  <si>
+    <t>3x NTCs /or RTDs</t>
+  </si>
+  <si>
+    <t>Temperatures sensing for tcs</t>
+  </si>
+  <si>
+    <t>Store map of earths magnetic field and map of stars, will use open startracker - https://github.com/UBNanosatLab/openstartracker- star database is 60MB (see hip_main.dat in repo) - magnetometer specs here - https://www.ncei.noaa.gov/products/world-magnetic-model?utm_source=chatgpt.com - file size 10kB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200MB </t>
+  </si>
+  <si>
+    <t>In progress!</t>
+  </si>
+  <si>
+    <t>https://app.diagrams.net/#G1EkgXl9bJNVBrBIp_C_mafJHwrpY2Lw2s#%7B%22pageId%22%3A%22j9GepUNVeoevYmeeWvKN%22%7D</t>
   </si>
 </sst>
 </file>
@@ -120,7 +226,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -139,8 +245,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -163,11 +293,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -178,11 +354,59 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -199,6 +423,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>44450</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>349586</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>89101</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43B0FF96-5ED4-7AAF-9E90-6D5FE43D486F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1873250" y="2070100"/>
+          <a:ext cx="6540836" cy="3911801"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,130 +737,379 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:E10"/>
+  <dimension ref="B2:F22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="103.54296875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="14.36328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="60.7265625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B3" s="2" t="s">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="F2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B3" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="E3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B4" s="18"/>
+      <c r="C4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B5" s="18"/>
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B6" s="18"/>
+      <c r="C6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7" s="18"/>
+      <c r="C7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B8" s="18"/>
+      <c r="C8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B9" s="19"/>
+      <c r="C9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B11" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B12" s="10"/>
+      <c r="C12" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B13" s="10"/>
+      <c r="C13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B14" s="10"/>
+      <c r="C14" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B16" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="11"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B17" s="21"/>
+      <c r="C17" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B18" s="15"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B20" s="15"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B21" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="12"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B3:B9"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B11:B14"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B8EADC9-8DE6-40C8-AB02-27F36E1859E1}">
+  <dimension ref="B3:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+        <v>25</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B10" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>18</v>
+        <v>29</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{863680D0-AE44-48B2-84CB-FA4BEB6B825E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{785FB57C-F006-4B53-A097-B592C90BAE7A}">
+  <dimension ref="E5:F5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="5" max="5" width="10.7265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="5:6" x14ac:dyDescent="0.35">
+      <c r="E5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D4DD80A-1E3B-43EE-A6AB-A0DBEA1B8E77}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added some mroe stuff on mcu
</commit_message>
<xml_diff>
--- a/ADCS/DesignCriteriaReview.xlsx
+++ b/ADCS/DesignCriteriaReview.xlsx
@@ -379,7 +379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -426,6 +426,12 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -446,15 +452,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -815,7 +812,7 @@
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="18" t="s">
         <v>33</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -832,7 +829,7 @@
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B4" s="17"/>
+      <c r="B4" s="19"/>
       <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
@@ -847,7 +844,7 @@
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B5" s="17"/>
+      <c r="B5" s="19"/>
       <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
@@ -862,7 +859,7 @@
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B6" s="17"/>
+      <c r="B6" s="19"/>
       <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
@@ -877,7 +874,7 @@
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B7" s="17"/>
+      <c r="B7" s="19"/>
       <c r="C7" s="4" t="s">
         <v>13</v>
       </c>
@@ -892,7 +889,7 @@
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B8" s="17"/>
+      <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
@@ -907,7 +904,7 @@
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="18"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="4" t="s">
         <v>47</v>
       </c>
@@ -929,7 +926,7 @@
       <c r="F10" s="8"/>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="23" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="4" t="s">
@@ -946,7 +943,7 @@
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B12" s="22"/>
+      <c r="B12" s="24"/>
       <c r="C12" s="4" t="s">
         <v>15</v>
       </c>
@@ -961,7 +958,7 @@
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B13" s="22"/>
+      <c r="B13" s="24"/>
       <c r="C13" s="4" t="s">
         <v>42</v>
       </c>
@@ -976,7 +973,7 @@
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B14" s="22"/>
+      <c r="B14" s="24"/>
       <c r="C14" s="10" t="s">
         <v>50</v>
       </c>
@@ -992,16 +989,16 @@
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="15"/>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="17" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1013,7 +1010,7 @@
       <c r="F16" s="8"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="21" t="s">
         <v>35</v>
       </c>
       <c r="C17" s="10" t="s">
@@ -1028,7 +1025,7 @@
       <c r="F17" s="9"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B18" s="23"/>
+      <c r="B18" s="22"/>
       <c r="C18" s="10" t="s">
         <v>65</v>
       </c>
@@ -1041,7 +1038,7 @@
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B19" s="20"/>
+      <c r="B19" s="22"/>
       <c r="C19" s="10" t="s">
         <v>51</v>
       </c>

</xml_diff>